<commit_message>
Mas recursos y paginas de nuevas maquinas
</commit_message>
<xml_diff>
--- a/Gestión de Producción/Corrección de entrega/CalculosCQS.xlsx
+++ b/Gestión de Producción/Corrección de entrega/CalculosCQS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Compa\Documents\2026A\APM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Compa\Documents\2026A\APM\Proyecto-APM---2026-1S\Gestión de Producción\Corrección de entrega\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B07824FC-2FA3-42D1-A5FE-DBCA82F88CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C2B548-1864-4ED7-AEF6-5C671F55C644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8D13AF91-1B32-462F-BA97-F85D34090091}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>Coca cola 2L, Quatro 1.75L, Sprote 1.5L</t>
   </si>
@@ -165,6 +165,48 @@
   </si>
   <si>
     <t>Este valor lo sacamos de algunas tesis, puesto que es bien dificil encontrar el valor el tiempo de ciclo real, entre otros valores que se necesitan para calcular este valor teoricamente</t>
+  </si>
+  <si>
+    <t>MLT</t>
+  </si>
+  <si>
+    <t>Soplado</t>
+  </si>
+  <si>
+    <t>Enjuagado</t>
+  </si>
+  <si>
+    <t>Llenado</t>
+  </si>
+  <si>
+    <t>Tapado</t>
+  </si>
+  <si>
+    <t>Etiquetado</t>
+  </si>
+  <si>
+    <t>Codificado</t>
+  </si>
+  <si>
+    <t>Embalaje</t>
+  </si>
+  <si>
+    <t>Paletizado</t>
+  </si>
+  <si>
+    <t>Almacenamiento</t>
+  </si>
+  <si>
+    <t>Tiempo(s)</t>
+  </si>
+  <si>
+    <t>Aqui tambien sumamos los tiempos de Setup</t>
+  </si>
+  <si>
+    <t>Al pasarlos a segundos</t>
+  </si>
+  <si>
+    <t>MLT (segundos)</t>
   </si>
 </sst>
 </file>
@@ -205,7 +247,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -218,13 +260,34 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -234,20 +297,20 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -320,8 +383,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>735106</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1344706</xdr:colOff>
       <xdr:row>75</xdr:row>
       <xdr:rowOff>146490</xdr:rowOff>
     </xdr:to>
@@ -686,6 +749,7 @@
     <col min="5" max="5" width="11.6640625" customWidth="1"/>
     <col min="6" max="6" width="17.21875" customWidth="1"/>
     <col min="7" max="7" width="10.44140625" customWidth="1"/>
+    <col min="8" max="8" width="20.44140625" customWidth="1"/>
     <col min="9" max="9" width="14.109375" customWidth="1"/>
     <col min="10" max="10" width="25.5546875" customWidth="1"/>
     <col min="11" max="11" width="58.88671875" customWidth="1"/>
@@ -743,12 +807,12 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="1"/>
+      <c r="A13" s="7"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -759,77 +823,77 @@
       <c r="A43" t="s">
         <v>10</v>
       </c>
-      <c r="B43" s="2" t="s">
+      <c r="B43" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D43" s="4">
+      <c r="D43" s="2">
         <v>352300000</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A78" s="3" t="s">
+      <c r="A78" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A79" s="3"/>
+      <c r="A79" s="5"/>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A80" s="3"/>
+      <c r="A80" s="5"/>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H82" s="3" t="s">
+      <c r="H82" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I82" s="3"/>
-      <c r="J82" s="3"/>
-      <c r="K82" s="3"/>
-      <c r="L82" s="3"/>
-      <c r="M82" s="3"/>
+      <c r="I82" s="5"/>
+      <c r="J82" s="5"/>
+      <c r="K82" s="5"/>
+      <c r="L82" s="5"/>
+      <c r="M82" s="5"/>
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>13</v>
       </c>
-      <c r="B83" s="5">
+      <c r="B83" s="3">
         <f>D43*0.76</f>
         <v>267748000</v>
       </c>
-      <c r="H83" s="3"/>
-      <c r="I83" s="3"/>
-      <c r="J83" s="3"/>
-      <c r="K83" s="3"/>
-      <c r="L83" s="3"/>
-      <c r="M83" s="3"/>
+      <c r="H83" s="5"/>
+      <c r="I83" s="5"/>
+      <c r="J83" s="5"/>
+      <c r="K83" s="5"/>
+      <c r="L83" s="5"/>
+      <c r="M83" s="5"/>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>14</v>
       </c>
-      <c r="B84" s="6">
+      <c r="B84">
         <f>B83*0.7</f>
         <v>187423600</v>
       </c>
-      <c r="H84" s="3"/>
-      <c r="I84" s="3"/>
-      <c r="J84" s="3"/>
-      <c r="K84" s="3"/>
-      <c r="L84" s="3"/>
-      <c r="M84" s="3"/>
+      <c r="H84" s="5"/>
+      <c r="I84" s="5"/>
+      <c r="J84" s="5"/>
+      <c r="K84" s="5"/>
+      <c r="L84" s="5"/>
+      <c r="M84" s="5"/>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="H85" s="3"/>
-      <c r="I85" s="3"/>
-      <c r="J85" s="3"/>
-      <c r="K85" s="3"/>
-      <c r="L85" s="3"/>
-      <c r="M85" s="3"/>
+      <c r="H85" s="5"/>
+      <c r="I85" s="5"/>
+      <c r="J85" s="5"/>
+      <c r="K85" s="5"/>
+      <c r="L85" s="5"/>
+      <c r="M85" s="5"/>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>15</v>
       </c>
-      <c r="B86" s="6">
+      <c r="B86">
         <f>B84/365</f>
         <v>513489.31506849313</v>
       </c>
@@ -850,7 +914,7 @@
       </c>
     </row>
     <row r="90" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="3" t="s">
+      <c r="A90" s="5" t="s">
         <v>17</v>
       </c>
       <c r="I90" t="s">
@@ -858,19 +922,19 @@
       </c>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A91" s="3"/>
+      <c r="A91" s="5"/>
       <c r="D91" t="s">
         <v>16</v>
       </c>
       <c r="F91" t="s">
         <v>23</v>
       </c>
-      <c r="J91" s="7" t="s">
+      <c r="J91" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A92" s="3"/>
+      <c r="A92" s="5"/>
       <c r="C92" t="s">
         <v>18</v>
       </c>
@@ -890,13 +954,13 @@
         <f>G92*0.5</f>
         <v>730181.80602739728</v>
       </c>
-      <c r="J92" s="7">
+      <c r="J92" s="4">
         <f>I92/2</f>
         <v>365090.90301369864</v>
       </c>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A93" s="3"/>
+      <c r="A93" s="5"/>
       <c r="C93" t="s">
         <v>19</v>
       </c>
@@ -916,13 +980,13 @@
         <f t="shared" ref="I93:I94" si="0">G93*0.5</f>
         <v>43810.908361643837</v>
       </c>
-      <c r="J93" s="7">
+      <c r="J93" s="4">
         <f>I93/1.75</f>
         <v>25034.804778082191</v>
       </c>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A94" s="3"/>
+      <c r="A94" s="5"/>
       <c r="C94" t="s">
         <v>20</v>
       </c>
@@ -942,19 +1006,19 @@
         <f t="shared" si="0"/>
         <v>43810.908361643837</v>
       </c>
-      <c r="J94" s="7">
+      <c r="J94" s="4">
         <f>I94/1.5</f>
         <v>29207.272241095892</v>
       </c>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A95" s="3"/>
+      <c r="A95" s="5"/>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A96" s="3"/>
+      <c r="A96" s="5"/>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A97" s="3"/>
+      <c r="A97" s="5"/>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
@@ -1001,7 +1065,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>32</v>
       </c>
@@ -1010,35 +1074,77 @@
         <v>296666.66666666669</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="123" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A123" s="3" t="s">
+    <row r="123" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B123" s="3"/>
-      <c r="C123" s="3"/>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A124" s="3"/>
-      <c r="B124" s="3"/>
-      <c r="C124" s="3"/>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A125" s="3"/>
-      <c r="B125" s="3"/>
-      <c r="C125" s="3"/>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B123" s="5"/>
+      <c r="C123" s="5"/>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A124" s="5"/>
+      <c r="B124" s="5"/>
+      <c r="C124" s="5"/>
+      <c r="H124" t="s">
+        <v>43</v>
+      </c>
+      <c r="I124" t="s">
+        <v>53</v>
+      </c>
+      <c r="K124" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A125" s="5"/>
+      <c r="B125" s="5"/>
+      <c r="C125" s="5"/>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H126" t="s">
+        <v>44</v>
+      </c>
+      <c r="I126">
+        <v>1.5</v>
+      </c>
+      <c r="K126">
+        <f>B7+(B8/60)</f>
+        <v>1.1666666666666667</v>
+      </c>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H128" t="s">
+        <v>45</v>
+      </c>
+      <c r="I128">
+        <v>2</v>
+      </c>
+      <c r="K128" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="E130">
         <f>5.3 *60</f>
         <v>318</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H130" t="s">
+        <v>46</v>
+      </c>
+      <c r="I130">
+        <v>0.18</v>
+      </c>
+      <c r="K130">
+        <f>K126*3600</f>
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>36</v>
       </c>
@@ -1049,7 +1155,23 @@
         <v>26</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H132" t="s">
+        <v>47</v>
+      </c>
+      <c r="I132">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H134" t="s">
+        <v>48</v>
+      </c>
+      <c r="I134">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>34</v>
       </c>
@@ -1058,15 +1180,54 @@
         <v>0.75280898876404501</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H136" t="s">
+        <v>49</v>
+      </c>
+      <c r="I136">
+        <v>0.5</v>
+      </c>
+      <c r="K136" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K137" s="8">
+        <f>K130+I144</f>
+        <v>4487.18</v>
+      </c>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H138" t="s">
+        <v>50</v>
+      </c>
+      <c r="I138">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H140" t="s">
+        <v>51</v>
+      </c>
+      <c r="I140">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>38</v>
       </c>
       <c r="B142">
         <v>3.8999999999999998E-3</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H142" t="s">
+        <v>52</v>
+      </c>
+      <c r="I142">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>39</v>
       </c>
@@ -1074,7 +1235,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>37</v>
       </c>
@@ -1082,6 +1243,10 @@
         <f>1-B142</f>
         <v>0.99609999999999999</v>
       </c>
+      <c r="I144">
+        <f>SUM(I126:I142)</f>
+        <v>287.18</v>
+      </c>
     </row>
     <row r="145" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
@@ -1093,26 +1258,26 @@
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A147" s="8" t="s">
+      <c r="A147" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B147" s="8"/>
-      <c r="C147" s="8"/>
-      <c r="D147" s="8"/>
-      <c r="E147" s="8"/>
-      <c r="F147" s="8"/>
-      <c r="G147" s="8"/>
-      <c r="H147" s="8"/>
+      <c r="B147" s="6"/>
+      <c r="C147" s="6"/>
+      <c r="D147" s="6"/>
+      <c r="E147" s="6"/>
+      <c r="F147" s="6"/>
+      <c r="G147" s="6"/>
+      <c r="H147" s="6"/>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A148" s="8"/>
-      <c r="B148" s="8"/>
-      <c r="C148" s="8"/>
-      <c r="D148" s="8"/>
-      <c r="E148" s="8"/>
-      <c r="F148" s="8"/>
-      <c r="G148" s="8"/>
-      <c r="H148" s="8"/>
+      <c r="A148" s="6"/>
+      <c r="B148" s="6"/>
+      <c r="C148" s="6"/>
+      <c r="D148" s="6"/>
+      <c r="E148" s="6"/>
+      <c r="F148" s="6"/>
+      <c r="G148" s="6"/>
+      <c r="H148" s="6"/>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A155" t="s">

</xml_diff>